<commit_message>
Excel init: activity workflows/priorities + minimal template
</commit_message>
<xml_diff>
--- a/src/main/resources/excel/system_init.xlsx
+++ b/src/main/resources/excel/system_init.xlsx
@@ -7,18 +7,21 @@
   </bookViews>
   <sheets>
     <sheet name="Status" r:id="rId3" sheetId="1"/>
-    <sheet name="Activity Type" r:id="rId4" sheetId="2"/>
-    <sheet name="Issue Type" r:id="rId5" sheetId="3"/>
-    <sheet name="Grid Entity" r:id="rId6" sheetId="4"/>
-    <sheet name="Page Entity" r:id="rId7" sheetId="5"/>
-    <sheet name="Activity" r:id="rId8" sheetId="6"/>
-    <sheet name="Issue" r:id="rId9" sheetId="7"/>
+    <sheet name="Workflow Entity" r:id="rId4" sheetId="2"/>
+    <sheet name="Workflow Status Relation" r:id="rId5" sheetId="3"/>
+    <sheet name="Activity Priority" r:id="rId6" sheetId="4"/>
+    <sheet name="Activity Type" r:id="rId7" sheetId="5"/>
+    <sheet name="Issue Type" r:id="rId8" sheetId="6"/>
+    <sheet name="Grid Entity" r:id="rId9" sheetId="7"/>
+    <sheet name="Page Entity" r:id="rId10" sheetId="8"/>
+    <sheet name="Activity" r:id="rId11" sheetId="9"/>
+    <sheet name="Issue" r:id="rId12" sheetId="10"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="153">
   <si>
     <t># Project Item Statuses (used by Activities, Issues, etc.)</t>
   </si>
@@ -65,10 +68,109 @@
     <t>#2E7D32</t>
   </si>
   <si>
+    <t># Workflows</t>
+  </si>
+  <si>
+    <t># Columns: Name (required)</t>
+  </si>
+  <si>
+    <t>Default Workflow</t>
+  </si>
+  <si>
+    <t># Workflow Status Transitions</t>
+  </si>
+  <si>
+    <t># Columns: Workflow (required), From Status (required), To Status (required), Is Initial Status, Roles (csv)</t>
+  </si>
+  <si>
+    <t>Workflow</t>
+  </si>
+  <si>
+    <t>From Status</t>
+  </si>
+  <si>
+    <t>To Status</t>
+  </si>
+  <si>
+    <t>Is Initial Status</t>
+  </si>
+  <si>
+    <t>Roles</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t># Activity Priorities</t>
+  </si>
+  <si>
+    <t># Columns: Name (required), Color, Sort Order, Priority Level, Is Default</t>
+  </si>
+  <si>
+    <t>Sort Order</t>
+  </si>
+  <si>
+    <t>Priority Level</t>
+  </si>
+  <si>
+    <t>Is Default</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>#B71C1C</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>#D32F2F</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
     <t># Activity Types</t>
   </si>
   <si>
-    <t># Columns: Name (required), Color</t>
+    <t># Columns: Name (required), Color, Sort Order, Level, Can Have Children, Non Deletable, Workflow</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>Can Have Children</t>
+  </si>
+  <si>
+    <t>Non Deletable</t>
   </si>
   <si>
     <t>Design</t>
@@ -77,6 +179,9 @@
     <t>#5E35B1</t>
   </si>
   <si>
+    <t>-1</t>
+  </si>
+  <si>
     <t>Development</t>
   </si>
   <si>
@@ -101,9 +206,6 @@
     <t>Bug</t>
   </si>
   <si>
-    <t>#D32F2F</t>
-  </si>
-  <si>
     <t>Improvement</t>
   </si>
   <si>
@@ -203,9 +305,6 @@
     <t>vaadin:tasks</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Issues Page</t>
   </si>
   <si>
@@ -245,13 +344,37 @@
     <t>Activity Type</t>
   </si>
   <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Start   Date</t>
+  </si>
+  <si>
     <t>Due   Date</t>
   </si>
   <si>
+    <t>Completion Date</t>
+  </si>
+  <si>
+    <t>Progress   %</t>
+  </si>
+  <si>
+    <t>Story Points</t>
+  </si>
+  <si>
     <t>Estimated   Hours</t>
   </si>
   <si>
     <t>Assigned To</t>
+  </si>
+  <si>
+    <t>Acceptance Criteria</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Results</t>
   </si>
   <si>
     <t>Design login screen</t>
@@ -262,43 +385,70 @@
 - validate error states</t>
   </si>
   <si>
+    <t>0</t>
+  </si>
+  <si>
     <t>8</t>
   </si>
   <si>
+    <t>UI matches specs and error states are covered</t>
+  </si>
+  <si>
+    <t>Created from Excel system init</t>
+  </si>
+  <si>
     <t>Implement authentication</t>
   </si>
   <si>
     <t>JWT-based auth implementation (access + refresh tokens)</t>
   </si>
   <si>
+    <t>35</t>
+  </si>
+  <si>
     <t>admin</t>
   </si>
   <si>
+    <t>Tokens validated; refresh rotation; logout invalidates tokens</t>
+  </si>
+  <si>
+    <t>Security review pending</t>
+  </si>
+  <si>
     <t>Write unit tests</t>
   </si>
   <si>
     <t>Cover authentication service with tests; include edge cases (Safari, iOS)</t>
   </si>
   <si>
+    <t>5</t>
+  </si>
+  <si>
     <t>4.5</t>
   </si>
   <si>
+    <t>Happy path + edge cases pass on CI</t>
+  </si>
+  <si>
+    <t>Use Playwright + unit test mix</t>
+  </si>
+  <si>
     <t>Document rollout plan</t>
   </si>
   <si>
     <t>Release notes + runbook update</t>
   </si>
   <si>
-    <t>2</t>
+    <t>Runbook includes rollback steps</t>
   </si>
   <si>
     <t>Verify formula date</t>
   </si>
   <si>
-    <t>Due date is generated via formula: E6+14 (safe POI-evaluable date arithmetic)</t>
-  </si>
-  <si>
-    <t>1</t>
+    <t>Due date is generated via formula: G7+14 (safe POI-evaluable date arithmetic)</t>
+  </si>
+  <si>
+    <t>Date formula evaluated on import</t>
   </si>
   <si>
     <t># Issue import template</t>
@@ -342,13 +492,49 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="21">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <i val="true"/>
+      <color indexed="23"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <i val="true"/>
+      <color indexed="23"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <i val="true"/>
+      <color indexed="23"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -468,7 +654,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
@@ -482,9 +668,15 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
 </styleSheet>
@@ -572,13 +764,138 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="86.87109375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="40.23046875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="6.4921875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="14.34375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="10.0390625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="22.40234375" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="11.359375" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="21">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="21">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="21">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="20">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s" s="20">
+        <v>104</v>
+      </c>
+      <c r="C4" t="s" s="20">
+        <v>105</v>
+      </c>
+      <c r="D4" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="E4" t="s" s="20">
+        <v>109</v>
+      </c>
+      <c r="F4" t="s" s="20">
+        <v>146</v>
+      </c>
+      <c r="G4" t="s" s="20">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>147</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>148</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="E5" t="n" s="22">
+        <v>45818.0</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>124</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>149</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>150</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="E6" t="n" s="22">
+        <v>45838.0</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>130</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>151</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>152</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E7" t="n" s="22">
+        <v>45843.0</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>136</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="27.95703125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="8.42578125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="22.9140625" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -595,40 +912,10 @@
       <c r="A3" t="s" s="3">
         <v>2</v>
       </c>
-      <c r="B3" t="s" s="3">
-        <v>4</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
         <v>17</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -638,61 +925,75 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="27.95703125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="8.3203125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="81.234375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="11.49609375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.3359375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="14.19140625" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="5.609375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="6">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="6">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="5">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s" s="5">
-        <v>4</v>
+        <v>21</v>
+      </c>
+      <c r="C3" t="s" s="5">
+        <v>22</v>
+      </c>
+      <c r="D3" t="s" s="5">
+        <v>23</v>
+      </c>
+      <c r="E3" t="s" s="5">
+        <v>24</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>27</v>
+        <v>6</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>25</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>29</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>32</v>
+        <v>10</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -701,6 +1002,406 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="56.17578125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="8.390625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.109375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="12.55859375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="9.44140625" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="8">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="8">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="7">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="7">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s" s="7">
+        <v>28</v>
+      </c>
+      <c r="D3" t="s" s="7">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s" s="7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="77.05078125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="8.42578125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.109375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="5.51953125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="16.99609375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="13.42578125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="15.19921875" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="10">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="10">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="9">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s" s="9">
+        <v>28</v>
+      </c>
+      <c r="D3" t="s" s="9">
+        <v>47</v>
+      </c>
+      <c r="E3" t="s" s="9">
+        <v>48</v>
+      </c>
+      <c r="F3" t="s" s="9">
+        <v>49</v>
+      </c>
+      <c r="G3" t="s" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="77.05078125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="8.3203125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.109375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="5.51953125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="16.99609375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="13.42578125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="15.19921875" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="12">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="12">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="11">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="11">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s" s="11">
+        <v>28</v>
+      </c>
+      <c r="D3" t="s" s="11">
+        <v>47</v>
+      </c>
+      <c r="E3" t="s" s="11">
+        <v>48</v>
+      </c>
+      <c r="F3" t="s" s="11">
+        <v>49</v>
+      </c>
+      <c r="G3" t="s" s="11">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -713,44 +1414,44 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="8">
-        <v>33</v>
+      <c r="A1" t="s" s="14">
+        <v>66</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="8">
-        <v>34</v>
+      <c r="A2" t="s" s="14">
+        <v>67</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="7">
+      <c r="A3" t="s" s="13">
         <v>2</v>
       </c>
-      <c r="B3" t="s" s="7">
-        <v>35</v>
-      </c>
-      <c r="C3" t="s" s="7">
-        <v>36</v>
-      </c>
-      <c r="D3" t="s" s="7">
-        <v>37</v>
-      </c>
-      <c r="E3" t="s" s="7">
-        <v>38</v>
+      <c r="B3" t="s" s="13">
+        <v>68</v>
+      </c>
+      <c r="C3" t="s" s="13">
+        <v>69</v>
+      </c>
+      <c r="D3" t="s" s="13">
+        <v>70</v>
+      </c>
+      <c r="E3" t="s" s="13">
+        <v>71</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>41</v>
+        <v>74</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>42</v>
+        <v>75</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>7</v>
@@ -758,16 +1459,16 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>43</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>45</v>
+        <v>78</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>42</v>
+        <v>75</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>7</v>
@@ -778,7 +1479,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -795,100 +1496,100 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="10">
-        <v>46</v>
+      <c r="A1" t="s" s="16">
+        <v>79</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="10">
-        <v>47</v>
+      <c r="A2" t="s" s="16">
+        <v>80</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="9">
+      <c r="A3" t="s" s="15">
         <v>2</v>
       </c>
-      <c r="B3" t="s" s="9">
-        <v>48</v>
-      </c>
-      <c r="C3" t="s" s="9">
-        <v>49</v>
-      </c>
-      <c r="D3" t="s" s="9">
-        <v>50</v>
-      </c>
-      <c r="E3" t="s" s="9">
-        <v>51</v>
-      </c>
-      <c r="F3" t="s" s="9">
+      <c r="B3" t="s" s="15">
+        <v>81</v>
+      </c>
+      <c r="C3" t="s" s="15">
+        <v>82</v>
+      </c>
+      <c r="D3" t="s" s="15">
+        <v>83</v>
+      </c>
+      <c r="E3" t="s" s="15">
+        <v>84</v>
+      </c>
+      <c r="F3" t="s" s="15">
         <v>5</v>
       </c>
-      <c r="G3" t="s" s="9">
-        <v>52</v>
-      </c>
-      <c r="H3" t="s" s="9">
-        <v>53</v>
-      </c>
-      <c r="I3" t="s" s="9">
-        <v>54</v>
+      <c r="G3" t="s" s="15">
+        <v>85</v>
+      </c>
+      <c r="H3" t="s" s="15">
+        <v>86</v>
+      </c>
+      <c r="I3" t="s" s="15">
+        <v>87</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>55</v>
+        <v>88</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>56</v>
+        <v>89</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>57</v>
+        <v>90</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>58</v>
+        <v>91</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>59</v>
+        <v>92</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>60</v>
+        <v>93</v>
       </c>
       <c r="G4" t="s" s="0">
         <v>13</v>
       </c>
       <c r="H4" t="s" s="0">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="I4" t="s" s="0">
-        <v>61</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>62</v>
+        <v>94</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>63</v>
+        <v>95</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>64</v>
+        <v>96</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>65</v>
+        <v>97</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>66</v>
+        <v>98</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>67</v>
+        <v>99</v>
       </c>
       <c r="G5" t="s" s="0">
         <v>13</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>43</v>
+        <v>76</v>
       </c>
       <c r="I5" t="s" s="0">
-        <v>61</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -896,303 +1597,319 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="80.453125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="64.56640625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="64.8671875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.3359375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="13.69921875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="10.0390625" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="16.34375" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="11.359375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="7.7265625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="10.7734375" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="10.0390625" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="15.640625" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="11.51953125" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" width="11.47265625" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="16.34375" customWidth="true" bestFit="true"/>
+    <col min="12" max="12" width="11.359375" customWidth="true" bestFit="true"/>
+    <col min="13" max="13" width="50.203125" customWidth="true" bestFit="true"/>
+    <col min="14" max="14" width="25.83984375" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" width="7.30078125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="12">
-        <v>68</v>
+      <c r="A1" t="s" s="18">
+        <v>100</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="12">
-        <v>69</v>
+      <c r="A2" t="s" s="18">
+        <v>101</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="12">
-        <v>70</v>
+      <c r="A3" t="s" s="18">
+        <v>102</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="12">
-        <v>71</v>
+      <c r="A4" t="s" s="18">
+        <v>103</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="11">
+      <c r="A5" t="s" s="17">
         <v>2</v>
       </c>
-      <c r="B5" t="s" s="11">
-        <v>72</v>
-      </c>
-      <c r="C5" t="s" s="11">
-        <v>73</v>
-      </c>
-      <c r="D5" t="s" s="11">
-        <v>74</v>
-      </c>
-      <c r="E5" t="s" s="11">
-        <v>75</v>
-      </c>
-      <c r="F5" t="s" s="11">
-        <v>76</v>
-      </c>
-      <c r="G5" t="s" s="11">
-        <v>77</v>
+      <c r="B5" t="s" s="17">
+        <v>104</v>
+      </c>
+      <c r="C5" t="s" s="17">
+        <v>105</v>
+      </c>
+      <c r="D5" t="s" s="17">
+        <v>106</v>
+      </c>
+      <c r="E5" t="s" s="17">
+        <v>107</v>
+      </c>
+      <c r="F5" t="s" s="17">
+        <v>108</v>
+      </c>
+      <c r="G5" t="s" s="17">
+        <v>109</v>
+      </c>
+      <c r="H5" t="s" s="17">
+        <v>110</v>
+      </c>
+      <c r="I5" t="s" s="17">
+        <v>111</v>
+      </c>
+      <c r="J5" t="s" s="17">
+        <v>112</v>
+      </c>
+      <c r="K5" t="s" s="17">
+        <v>113</v>
+      </c>
+      <c r="L5" t="s" s="17">
+        <v>114</v>
+      </c>
+      <c r="M5" t="s" s="17">
+        <v>115</v>
+      </c>
+      <c r="N5" t="s" s="17">
+        <v>116</v>
+      </c>
+      <c r="O5" t="s" s="17">
+        <v>117</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>78</v>
+        <v>118</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>79</v>
+        <v>119</v>
       </c>
       <c r="C6" t="s" s="0">
         <v>6</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="E6" t="n" s="13">
+        <v>50</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>45818.0</v>
+      </c>
+      <c r="G6" s="19" t="n">
         <v>45823.0</v>
       </c>
-      <c r="F6" t="s" s="0">
-        <v>80</v>
-      </c>
-      <c r="G6" t="s" s="0">
-        <v>61</v>
+      <c r="H6" s="19"/>
+      <c r="I6" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="J6" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="K6" t="s" s="0">
+        <v>121</v>
+      </c>
+      <c r="L6" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="M6" t="s" s="0">
+        <v>122</v>
+      </c>
+      <c r="N6" t="s" s="0">
+        <v>123</v>
+      </c>
+      <c r="O6" t="s" s="0">
+        <v>25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>81</v>
+        <v>124</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>82</v>
+        <v>125</v>
       </c>
       <c r="C7" t="s" s="0">
         <v>10</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="E7" t="n" s="13">
+        <v>53</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>45820.0</v>
+      </c>
+      <c r="G7" s="19" t="n">
         <v>45828.0</v>
       </c>
-      <c r="F7" s="0">
+      <c r="H7" s="19"/>
+      <c r="I7" t="s" s="0">
+        <v>126</v>
+      </c>
+      <c r="J7" t="s" s="0">
+        <v>121</v>
+      </c>
+      <c r="K7" s="0">
         <f>4+4</f>
       </c>
-      <c r="G7" t="s" s="0">
-        <v>83</v>
+      <c r="L7" t="s" s="0">
+        <v>127</v>
+      </c>
+      <c r="M7" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="N7" t="s" s="0">
+        <v>129</v>
+      </c>
+      <c r="O7" t="s" s="0">
+        <v>25</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>84</v>
+        <v>130</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>85</v>
+        <v>131</v>
       </c>
       <c r="C8" t="s" s="0">
         <v>6</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="E8" t="n" s="13">
+        <v>55</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>45823.0</v>
+      </c>
+      <c r="G8" s="19" t="n">
         <v>45833.0</v>
       </c>
-      <c r="F8" t="s" s="0">
-        <v>86</v>
-      </c>
-      <c r="G8" t="s" s="0">
-        <v>83</v>
+      <c r="H8" s="19"/>
+      <c r="I8" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="J8" t="s" s="0">
+        <v>132</v>
+      </c>
+      <c r="K8" t="s" s="0">
+        <v>133</v>
+      </c>
+      <c r="L8" t="s" s="0">
+        <v>127</v>
+      </c>
+      <c r="M8" t="s" s="0">
+        <v>134</v>
+      </c>
+      <c r="N8" t="s" s="0">
+        <v>135</v>
+      </c>
+      <c r="O8" t="s" s="0">
+        <v>25</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>87</v>
+        <v>136</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>88</v>
+        <v>137</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="E9" t="n" s="13">
+        <v>57</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>45824.0</v>
+      </c>
+      <c r="G9" s="19" t="n">
         <v>45826.0</v>
       </c>
-      <c r="F9" t="s" s="0">
-        <v>89</v>
-      </c>
-      <c r="G9" t="s" s="0">
-        <v>61</v>
+      <c r="H9" s="19"/>
+      <c r="I9" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="J9" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="K9" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="L9" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="M9" t="s" s="0">
+        <v>138</v>
+      </c>
+      <c r="N9" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="O9" t="s" s="0">
+        <v>25</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>90</v>
+        <v>139</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>91</v>
+        <v>140</v>
       </c>
       <c r="C10" t="s" s="0">
         <v>6</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="E10" t="n" s="13">
-        <f>E6+14</f>
+        <v>55</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="F10" s="19" t="n">
         <v>45809.0</v>
       </c>
-      <c r="F10" t="s" s="0">
-        <v>92</v>
-      </c>
-      <c r="G10" t="s" s="0">
-        <v>61</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <cols>
-    <col min="1" max="1" width="86.87109375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="40.23046875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="6.4921875" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="14.34375" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="10.0390625" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="22.40234375" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="11.359375" customWidth="true" bestFit="true"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="15">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="15">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="15">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="14">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s" s="14">
-        <v>72</v>
-      </c>
-      <c r="C4" t="s" s="14">
-        <v>73</v>
-      </c>
-      <c r="D4" t="s" s="14">
-        <v>96</v>
-      </c>
-      <c r="E4" t="s" s="14">
-        <v>75</v>
-      </c>
-      <c r="F4" t="s" s="14">
-        <v>97</v>
-      </c>
-      <c r="G4" t="s" s="14">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>98</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>99</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>26</v>
-      </c>
-      <c r="E5" t="n" s="16">
-        <v>45818.0</v>
-      </c>
-      <c r="F5" t="s" s="0">
-        <v>81</v>
-      </c>
-      <c r="G5" t="s" s="0">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>100</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="C6" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>28</v>
-      </c>
-      <c r="E6" t="n" s="16">
-        <v>45838.0</v>
-      </c>
-      <c r="F6" t="s" s="0">
-        <v>84</v>
-      </c>
-      <c r="G6" t="s" s="0">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
-        <v>102</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>103</v>
-      </c>
-      <c r="C7" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="E7" t="n" s="16">
-        <v>45843.0</v>
-      </c>
-      <c r="F7" t="s" s="0">
-        <v>87</v>
-      </c>
-      <c r="G7" t="s" s="0">
-        <v>61</v>
+      <c r="G10" s="19" t="n">
+        <f>G7+14</f>
+        <v>45809.0</v>
+      </c>
+      <c r="H10" s="19"/>
+      <c r="I10" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="J10" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="K10" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="L10" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="M10" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="N10" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="O10" t="s" s="0">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expand Excel system_init imports
</commit_message>
<xml_diff>
--- a/src/main/resources/excel/system_init.xlsx
+++ b/src/main/resources/excel/system_init.xlsx
@@ -14,21 +14,28 @@
     <sheet name="Issue Type" r:id="rId8" sheetId="6"/>
     <sheet name="Meeting Type" r:id="rId9" sheetId="7"/>
     <sheet name="Decision Type" r:id="rId10" sheetId="8"/>
-    <sheet name="Grid Entity" r:id="rId11" sheetId="9"/>
-    <sheet name="Page Entity" r:id="rId12" sheetId="10"/>
-    <sheet name="Activity" r:id="rId13" sheetId="11"/>
-    <sheet name="Issue" r:id="rId14" sheetId="12"/>
-    <sheet name="Meeting" r:id="rId15" sheetId="13"/>
-    <sheet name="Decision" r:id="rId16" sheetId="14"/>
-    <sheet name="Comment" r:id="rId17" sheetId="15"/>
-    <sheet name="Link" r:id="rId18" sheetId="16"/>
-    <sheet name="Agile Parent Relation" r:id="rId19" sheetId="17"/>
+    <sheet name="User Story Type" r:id="rId11" sheetId="9"/>
+    <sheet name="Sprint Type" r:id="rId12" sheetId="10"/>
+    <sheet name="Ticket Priority" r:id="rId13" sheetId="11"/>
+    <sheet name="Ticket Type" r:id="rId14" sheetId="12"/>
+    <sheet name="Grid Entity" r:id="rId15" sheetId="13"/>
+    <sheet name="Page Entity" r:id="rId16" sheetId="14"/>
+    <sheet name="Activity" r:id="rId17" sheetId="15"/>
+    <sheet name="Issue" r:id="rId18" sheetId="16"/>
+    <sheet name="User Story" r:id="rId19" sheetId="17"/>
+    <sheet name="Sprint" r:id="rId20" sheetId="18"/>
+    <sheet name="Meeting" r:id="rId21" sheetId="19"/>
+    <sheet name="Decision" r:id="rId22" sheetId="20"/>
+    <sheet name="Ticket" r:id="rId23" sheetId="21"/>
+    <sheet name="Comment" r:id="rId24" sheetId="22"/>
+    <sheet name="Link" r:id="rId25" sheetId="23"/>
+    <sheet name="Agile Parent Relation" r:id="rId26" sheetId="24"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="303">
   <si>
     <t># Project Item Statuses (used by Activities, Issues, etc.)</t>
   </si>
@@ -267,6 +274,39 @@
     <t>Budget</t>
   </si>
   <si>
+    <t># User Story Types</t>
+  </si>
+  <si>
+    <t>Story</t>
+  </si>
+  <si>
+    <t>#1F8EFA</t>
+  </si>
+  <si>
+    <t>Spike</t>
+  </si>
+  <si>
+    <t># Sprint Types</t>
+  </si>
+  <si>
+    <t>Sprint</t>
+  </si>
+  <si>
+    <t>#8377C5</t>
+  </si>
+  <si>
+    <t># Ticket Priorities</t>
+  </si>
+  <si>
+    <t># Ticket Types</t>
+  </si>
+  <si>
+    <t>Support</t>
+  </si>
+  <si>
+    <t>#3A5791</t>
+  </si>
+  <si>
     <t># Grid Entities (view configuration)</t>
   </si>
   <si>
@@ -306,6 +346,36 @@
     <t>id,name,status,dueDate,assignedTo,linkedActivity</t>
   </si>
   <si>
+    <t>User Stories Grid</t>
+  </si>
+  <si>
+    <t>CUserStoryService</t>
+  </si>
+  <si>
+    <t>id,name,status,dueDate,assignedTo,storyPoint</t>
+  </si>
+  <si>
+    <t>Tickets Grid</t>
+  </si>
+  <si>
+    <t>CTicketService</t>
+  </si>
+  <si>
+    <t>id,name,status,dueDate,priority,assignedTo</t>
+  </si>
+  <si>
+    <t>Sprints Grid</t>
+  </si>
+  <si>
+    <t>CSprintService</t>
+  </si>
+  <si>
+    <t>id,name,status,startDate,endDate,velocity</t>
+  </si>
+  <si>
+    <t>name,status,startDate,endDate</t>
+  </si>
+  <si>
     <t># Page Entities (navigation pages)</t>
   </si>
   <si>
@@ -367,6 +437,60 @@
   </si>
   <si>
     <t>vaadin:bug</t>
+  </si>
+  <si>
+    <t>User Stories Page</t>
+  </si>
+  <si>
+    <t>Project.User Stories (Excel)</t>
+  </si>
+  <si>
+    <t>10.203</t>
+  </si>
+  <si>
+    <t>User Stories (Excel)</t>
+  </si>
+  <si>
+    <t>CPageServiceUserStory</t>
+  </si>
+  <si>
+    <t>vaadin:comment</t>
+  </si>
+  <si>
+    <t>Tickets Page</t>
+  </si>
+  <si>
+    <t>Project.Tickets (Excel)</t>
+  </si>
+  <si>
+    <t>10.204</t>
+  </si>
+  <si>
+    <t>Tickets (Excel)</t>
+  </si>
+  <si>
+    <t>CPageServiceTicket</t>
+  </si>
+  <si>
+    <t>vaadin:ticket</t>
+  </si>
+  <si>
+    <t>Sprints Page</t>
+  </si>
+  <si>
+    <t>Project.Sprints (Excel)</t>
+  </si>
+  <si>
+    <t>10.205</t>
+  </si>
+  <si>
+    <t>Sprints (Excel)</t>
+  </si>
+  <si>
+    <t>CPageServiceSprint</t>
+  </si>
+  <si>
+    <t>vaadin:calendar-clock</t>
   </si>
   <si>
     <t># Activity import template</t>
@@ -531,6 +655,88 @@
     <t>Add CSV export to all report pages</t>
   </si>
   <si>
+    <t># User story import sheet (project items)</t>
+  </si>
+  <si>
+    <t># Columns: Name (required), Description, Status, User Story Type, Start Date, Due Date, Completion Date, Progress %, Story Points, Assigned To, Acceptance Criteria, Notes, Results</t>
+  </si>
+  <si>
+    <t>User Story Type</t>
+  </si>
+  <si>
+    <t>Start Date</t>
+  </si>
+  <si>
+    <t>Due Date</t>
+  </si>
+  <si>
+    <t>Progress %</t>
+  </si>
+  <si>
+    <t>As an account owner I can enroll MFA for my workspace admins</t>
+  </si>
+  <si>
+    <t>Security: require MFA enrollment and enforce it for admins.</t>
+  </si>
+  <si>
+    <t>2025-06-01</t>
+  </si>
+  <si>
+    <t>2025-06-30</t>
+  </si>
+  <si>
+    <t>- Must support TOTP
+- Recovery codes
+- Admin enforcement</t>
+  </si>
+  <si>
+    <t>Sync with SSO roadmap</t>
+  </si>
+  <si>
+    <t># Sprint import sheet (project items)</t>
+  </si>
+  <si>
+    <t># Columns: Name (required), Description, Status, Sprint Type, Start Date, End Date (required by domain rules), Sprint Goal, Definition of Done, Retrospective Notes, Color, Velocity</t>
+  </si>
+  <si>
+    <t>Sprint Type</t>
+  </si>
+  <si>
+    <t>End Date</t>
+  </si>
+  <si>
+    <t>Sprint Goal</t>
+  </si>
+  <si>
+    <t>Definition of Done</t>
+  </si>
+  <si>
+    <t>Retrospective Notes</t>
+  </si>
+  <si>
+    <t>Velocity</t>
+  </si>
+  <si>
+    <t>Sprint 24</t>
+  </si>
+  <si>
+    <t>Identity hardening sprint.</t>
+  </si>
+  <si>
+    <t>2025-06-10</t>
+  </si>
+  <si>
+    <t>2025-06-24</t>
+  </si>
+  <si>
+    <t>MFA enrollment for admins</t>
+  </si>
+  <si>
+    <t>- Build
+- Test
+- Document</t>
+  </si>
+  <si>
     <t># Meeting import sheet (project items)</t>
   </si>
   <si>
@@ -540,15 +746,9 @@
     <t>Meeting Type</t>
   </si>
   <si>
-    <t>Start Date</t>
-  </si>
-  <si>
     <t>Start Time</t>
   </si>
   <si>
-    <t>End Date</t>
-  </si>
-  <si>
     <t>End Time</t>
   </si>
   <si>
@@ -577,9 +777,6 @@
   </si>
   <si>
     <t>Plan sprint scope and break down identity rollout work</t>
-  </si>
-  <si>
-    <t>2025-06-10</t>
   </si>
   <si>
     <t>09:00</t>
@@ -632,6 +829,33 @@
     <t>2025-06-25T09:00</t>
   </si>
   <si>
+    <t># Ticket import sheet (project items)</t>
+  </si>
+  <si>
+    <t># Columns: Name (required), Description, Status, Ticket Type, Due Date, Priority, Assigned To, Context Information, Result</t>
+  </si>
+  <si>
+    <t>Ticket Type</t>
+  </si>
+  <si>
+    <t>Context Information</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>MFA enrollment fails for some admins</t>
+  </si>
+  <si>
+    <t>Investigate edge cases in enrollment flow and fix.</t>
+  </si>
+  <si>
+    <t>2025-06-20</t>
+  </si>
+  <si>
+    <t>Safari 17 + WebAuthn disabled</t>
+  </si>
+  <si>
     <t># Comments (child entities)
 # Owner Type/Name resolve entities by name in the active project</t>
   </si>
@@ -672,6 +896,18 @@
     <t>Compare SSO support and audit logging.</t>
   </si>
   <si>
+    <t>User Story</t>
+  </si>
+  <si>
+    <t>Capture unhappy-path cases and browser constraints.</t>
+  </si>
+  <si>
+    <t>Ticket</t>
+  </si>
+  <si>
+    <t>Reproduce on Safari and document workaround.</t>
+  </si>
+  <si>
     <t># Links (child entities)
 # Bidirectional=true creates a reverse link if target supports links</t>
   </si>
@@ -703,6 +939,12 @@
     <t>Implementation must follow the provider choice</t>
   </si>
   <si>
+    <t>Relates To</t>
+  </si>
+  <si>
+    <t>Ticket contributes evidence and repro steps for the story</t>
+  </si>
+  <si>
     <t># Agile hierarchy links (Owner -&gt; Parent)
 # Parent may be blank to explicitly mark the owner as a root item</t>
   </si>
@@ -714,12 +956,6 @@
   </si>
   <si>
     <t>Parent Name</t>
-  </si>
-  <si>
-    <t>User Story</t>
-  </si>
-  <si>
-    <t>As an account owner I can enroll MFA for my workspace admins</t>
   </si>
 </sst>
 </file>
@@ -729,13 +965,97 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="35">
+  <fonts count="49">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <i val="true"/>
+      <color indexed="23"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <i val="true"/>
+      <color indexed="23"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <i val="true"/>
+      <color indexed="23"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <i val="true"/>
+      <color indexed="23"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <i val="true"/>
+      <color indexed="23"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <i val="true"/>
+      <color indexed="23"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <i val="true"/>
+      <color indexed="23"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -975,7 +1295,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
@@ -999,20 +1319,34 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="0" fontId="23" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="0" fontId="25" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="27" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="29" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="0" fontId="31" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="0" fontId="33" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="39" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="41" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="43" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="45" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="47" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -1101,28 +1435,26 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="92.71484375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="20.0859375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.48828125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="13.875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="17.8515625" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="11.05859375" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="22.27734375" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="12.171875" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="7.98046875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="77.05078125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="8.1484375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.109375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="5.51953125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="16.99609375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="13.42578125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="17.5703125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="20">
-        <v>92</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="20">
-        <v>93</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3">
@@ -1130,86 +1462,45 @@
         <v>2</v>
       </c>
       <c r="B3" t="s" s="19">
-        <v>94</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s" s="19">
-        <v>95</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s" s="19">
-        <v>96</v>
+        <v>48</v>
       </c>
       <c r="E3" t="s" s="19">
-        <v>97</v>
+        <v>49</v>
       </c>
       <c r="F3" t="s" s="19">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="G3" t="s" s="19">
-        <v>98</v>
-      </c>
-      <c r="H3" t="s" s="19">
-        <v>99</v>
-      </c>
-      <c r="I3" t="s" s="19">
-        <v>100</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>102</v>
+        <v>85</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>103</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>104</v>
+        <v>53</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>105</v>
+        <v>7</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>106</v>
+        <v>7</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="H4" t="s" s="0">
-        <v>85</v>
-      </c>
-      <c r="I4" t="s" s="0">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>107</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>108</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>109</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>110</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>111</v>
-      </c>
-      <c r="F5" t="s" s="0">
-        <v>112</v>
-      </c>
-      <c r="G5" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="H5" t="s" s="0">
-        <v>89</v>
-      </c>
-      <c r="I5" t="s" s="0">
-        <v>26</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -1218,6 +1509,533 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="56.17578125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="8.3203125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.109375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="12.55859375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="9.44140625" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="22">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="22">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="21">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="21">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s" s="21">
+        <v>29</v>
+      </c>
+      <c r="D3" t="s" s="21">
+        <v>30</v>
+      </c>
+      <c r="E3" t="s" s="21">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="77.05078125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="8.16015625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.109375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="5.51953125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="16.99609375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="13.42578125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="17.5703125" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="24">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="24">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="23">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="23">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s" s="23">
+        <v>29</v>
+      </c>
+      <c r="D3" t="s" s="23">
+        <v>48</v>
+      </c>
+      <c r="E3" t="s" s="23">
+        <v>49</v>
+      </c>
+      <c r="F3" t="s" s="23">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s" s="23">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="92.55078125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="16.671875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="41.7109375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="26.69140625" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="9.7734375" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="26">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="26">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="25">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="25">
+        <v>92</v>
+      </c>
+      <c r="C3" t="s" s="25">
+        <v>93</v>
+      </c>
+      <c r="D3" t="s" s="25">
+        <v>94</v>
+      </c>
+      <c r="E3" t="s" s="25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>101</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>103</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>105</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>107</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>109</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>110</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>111</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>112</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="92.71484375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="22.7265625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.48828125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="16.51171875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="20.03515625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="18.63671875" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="22.27734375" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="14.8125" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="7.98046875" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="28">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="28">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="27">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="27">
+        <v>115</v>
+      </c>
+      <c r="C3" t="s" s="27">
+        <v>116</v>
+      </c>
+      <c r="D3" t="s" s="27">
+        <v>117</v>
+      </c>
+      <c r="E3" t="s" s="27">
+        <v>118</v>
+      </c>
+      <c r="F3" t="s" s="27">
+        <v>5</v>
+      </c>
+      <c r="G3" t="s" s="27">
+        <v>119</v>
+      </c>
+      <c r="H3" t="s" s="27">
+        <v>120</v>
+      </c>
+      <c r="I3" t="s" s="27">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>122</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>123</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>124</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>125</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>126</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>127</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>129</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>130</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>131</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>132</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>133</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="I5" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>134</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>135</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>136</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>137</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>138</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>139</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H6" t="s" s="0">
+        <v>103</v>
+      </c>
+      <c r="I6" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>140</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>142</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>143</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>144</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>145</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H7" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="I7" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>146</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>147</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>148</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>149</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>150</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>151</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H8" t="s" s="0">
+        <v>109</v>
+      </c>
+      <c r="I8" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:O10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -1240,78 +2058,78 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="22">
-        <v>113</v>
+      <c r="A1" t="s" s="30">
+        <v>152</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="22">
-        <v>114</v>
+      <c r="A2" t="s" s="30">
+        <v>153</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="22">
-        <v>115</v>
+      <c r="A3" t="s" s="30">
+        <v>154</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="22">
-        <v>116</v>
+      <c r="A4" t="s" s="30">
+        <v>155</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="21">
+      <c r="A5" t="s" s="29">
         <v>2</v>
       </c>
-      <c r="B5" t="s" s="21">
-        <v>117</v>
-      </c>
-      <c r="C5" t="s" s="21">
-        <v>118</v>
-      </c>
-      <c r="D5" t="s" s="21">
-        <v>119</v>
-      </c>
-      <c r="E5" t="s" s="21">
-        <v>120</v>
-      </c>
-      <c r="F5" t="s" s="21">
-        <v>121</v>
-      </c>
-      <c r="G5" t="s" s="21">
-        <v>122</v>
-      </c>
-      <c r="H5" t="s" s="21">
-        <v>123</v>
-      </c>
-      <c r="I5" t="s" s="21">
-        <v>124</v>
-      </c>
-      <c r="J5" t="s" s="21">
-        <v>125</v>
-      </c>
-      <c r="K5" t="s" s="21">
-        <v>126</v>
-      </c>
-      <c r="L5" t="s" s="21">
-        <v>127</v>
-      </c>
-      <c r="M5" t="s" s="21">
-        <v>128</v>
-      </c>
-      <c r="N5" t="s" s="21">
-        <v>129</v>
-      </c>
-      <c r="O5" t="s" s="21">
-        <v>130</v>
+      <c r="B5" t="s" s="29">
+        <v>156</v>
+      </c>
+      <c r="C5" t="s" s="29">
+        <v>157</v>
+      </c>
+      <c r="D5" t="s" s="29">
+        <v>158</v>
+      </c>
+      <c r="E5" t="s" s="29">
+        <v>159</v>
+      </c>
+      <c r="F5" t="s" s="29">
+        <v>160</v>
+      </c>
+      <c r="G5" t="s" s="29">
+        <v>161</v>
+      </c>
+      <c r="H5" t="s" s="29">
+        <v>162</v>
+      </c>
+      <c r="I5" t="s" s="29">
+        <v>163</v>
+      </c>
+      <c r="J5" t="s" s="29">
+        <v>164</v>
+      </c>
+      <c r="K5" t="s" s="29">
+        <v>165</v>
+      </c>
+      <c r="L5" t="s" s="29">
+        <v>166</v>
+      </c>
+      <c r="M5" t="s" s="29">
+        <v>167</v>
+      </c>
+      <c r="N5" t="s" s="29">
+        <v>168</v>
+      </c>
+      <c r="O5" t="s" s="29">
+        <v>169</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>131</v>
+        <v>170</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>132</v>
+        <v>171</v>
       </c>
       <c r="C6" t="s" s="0">
         <v>6</v>
@@ -1322,30 +2140,30 @@
       <c r="E6" t="s" s="0">
         <v>36</v>
       </c>
-      <c r="F6" s="23" t="n">
+      <c r="F6" s="31" t="n">
         <v>45818.0</v>
       </c>
-      <c r="G6" s="23" t="n">
+      <c r="G6" s="31" t="n">
         <v>45823.0</v>
       </c>
-      <c r="H6" s="23"/>
+      <c r="H6" s="31"/>
       <c r="I6" t="s" s="0">
-        <v>133</v>
+        <v>172</v>
       </c>
       <c r="J6" t="s" s="0">
         <v>42</v>
       </c>
       <c r="K6" t="s" s="0">
-        <v>134</v>
+        <v>173</v>
       </c>
       <c r="L6" t="s" s="0">
         <v>26</v>
       </c>
       <c r="M6" t="s" s="0">
-        <v>135</v>
+        <v>174</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>136</v>
+        <v>175</v>
       </c>
       <c r="O6" t="s" s="0">
         <v>26</v>
@@ -1353,10 +2171,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>137</v>
+        <v>176</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>138</v>
+        <v>177</v>
       </c>
       <c r="C7" t="s" s="0">
         <v>10</v>
@@ -1367,30 +2185,30 @@
       <c r="E7" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="F7" s="23" t="n">
+      <c r="F7" s="31" t="n">
         <v>45820.0</v>
       </c>
-      <c r="G7" s="23" t="n">
+      <c r="G7" s="31" t="n">
         <v>45828.0</v>
       </c>
-      <c r="H7" s="23"/>
+      <c r="H7" s="31"/>
       <c r="I7" t="s" s="0">
-        <v>139</v>
+        <v>178</v>
       </c>
       <c r="J7" t="s" s="0">
-        <v>134</v>
+        <v>173</v>
       </c>
       <c r="K7" s="0">
         <f>4+4</f>
       </c>
       <c r="L7" t="s" s="0">
-        <v>140</v>
+        <v>179</v>
       </c>
       <c r="M7" t="s" s="0">
-        <v>141</v>
+        <v>180</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>142</v>
+        <v>181</v>
       </c>
       <c r="O7" t="s" s="0">
         <v>26</v>
@@ -1398,10 +2216,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>143</v>
+        <v>182</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>144</v>
+        <v>183</v>
       </c>
       <c r="C8" t="s" s="0">
         <v>6</v>
@@ -1412,30 +2230,30 @@
       <c r="E8" t="s" s="0">
         <v>40</v>
       </c>
-      <c r="F8" s="23" t="n">
+      <c r="F8" s="31" t="n">
         <v>45823.0</v>
       </c>
-      <c r="G8" s="23" t="n">
+      <c r="G8" s="31" t="n">
         <v>45833.0</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="31"/>
       <c r="I8" t="s" s="0">
-        <v>133</v>
+        <v>172</v>
       </c>
       <c r="J8" t="s" s="0">
-        <v>145</v>
+        <v>184</v>
       </c>
       <c r="K8" t="s" s="0">
-        <v>146</v>
+        <v>185</v>
       </c>
       <c r="L8" t="s" s="0">
-        <v>140</v>
+        <v>179</v>
       </c>
       <c r="M8" t="s" s="0">
-        <v>147</v>
+        <v>186</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>148</v>
+        <v>187</v>
       </c>
       <c r="O8" t="s" s="0">
         <v>26</v>
@@ -1443,10 +2261,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>149</v>
+        <v>188</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>150</v>
+        <v>189</v>
       </c>
       <c r="C9" t="s" s="0">
         <v>26</v>
@@ -1457,15 +2275,15 @@
       <c r="E9" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="31" t="n">
         <v>45824.0</v>
       </c>
-      <c r="G9" s="23" t="n">
+      <c r="G9" s="31" t="n">
         <v>45826.0</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="31"/>
       <c r="I9" t="s" s="0">
-        <v>133</v>
+        <v>172</v>
       </c>
       <c r="J9" t="s" s="0">
         <v>39</v>
@@ -1477,7 +2295,7 @@
         <v>26</v>
       </c>
       <c r="M9" t="s" s="0">
-        <v>151</v>
+        <v>190</v>
       </c>
       <c r="N9" t="s" s="0">
         <v>26</v>
@@ -1488,10 +2306,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>153</v>
+        <v>192</v>
       </c>
       <c r="C10" t="s" s="0">
         <v>6</v>
@@ -1502,16 +2320,16 @@
       <c r="E10" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="31" t="n">
         <v>45809.0</v>
       </c>
-      <c r="G10" s="23" t="n">
+      <c r="G10" s="31" t="n">
         <f>G7+14</f>
         <v>45809.0</v>
       </c>
-      <c r="H10" s="23"/>
+      <c r="H10" s="31"/>
       <c r="I10" t="s" s="0">
-        <v>133</v>
+        <v>172</v>
       </c>
       <c r="J10" t="s" s="0">
         <v>35</v>
@@ -1523,7 +2341,7 @@
         <v>26</v>
       </c>
       <c r="M10" t="s" s="0">
-        <v>154</v>
+        <v>193</v>
       </c>
       <c r="N10" t="s" s="0">
         <v>26</v>
@@ -1537,7 +2355,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -1552,49 +2370,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="25">
-        <v>155</v>
+      <c r="A1" t="s" s="33">
+        <v>194</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="25">
+      <c r="A2" t="s" s="33">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="33">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="32">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s" s="32">
         <v>156</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="25">
+      <c r="C4" t="s" s="32">
         <v>157</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="24">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s" s="24">
-        <v>117</v>
-      </c>
-      <c r="C4" t="s" s="24">
-        <v>118</v>
-      </c>
-      <c r="D4" t="s" s="24">
-        <v>158</v>
-      </c>
-      <c r="E4" t="s" s="24">
-        <v>122</v>
-      </c>
-      <c r="F4" t="s" s="24">
-        <v>159</v>
-      </c>
-      <c r="G4" t="s" s="24">
-        <v>127</v>
+      <c r="D4" t="s" s="32">
+        <v>197</v>
+      </c>
+      <c r="E4" t="s" s="32">
+        <v>161</v>
+      </c>
+      <c r="F4" t="s" s="32">
+        <v>198</v>
+      </c>
+      <c r="G4" t="s" s="32">
+        <v>166</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>160</v>
+        <v>199</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>161</v>
+        <v>200</v>
       </c>
       <c r="C5" t="s" s="0">
         <v>6</v>
@@ -1602,22 +2420,22 @@
       <c r="D5" t="s" s="0">
         <v>61</v>
       </c>
-      <c r="E5" t="n" s="26">
+      <c r="E5" t="n" s="34">
         <v>45818.0</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>137</v>
+        <v>176</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>140</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>162</v>
+        <v>201</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>163</v>
+        <v>202</v>
       </c>
       <c r="C6" t="s" s="0">
         <v>6</v>
@@ -1625,22 +2443,22 @@
       <c r="D6" t="s" s="0">
         <v>62</v>
       </c>
-      <c r="E6" t="n" s="26">
+      <c r="E6" t="n" s="34">
         <v>45838.0</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>143</v>
+        <v>182</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>140</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>164</v>
+        <v>203</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>165</v>
+        <v>204</v>
       </c>
       <c r="C7" t="s" s="0">
         <v>6</v>
@@ -1648,11 +2466,11 @@
       <c r="D7" t="s" s="0">
         <v>65</v>
       </c>
-      <c r="E7" t="n" s="26">
+      <c r="E7" t="n" s="34">
         <v>45843.0</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>149</v>
+        <v>188</v>
       </c>
       <c r="G7" t="s" s="0">
         <v>26</v>
@@ -1663,7 +2481,227 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:M4"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="138.90234375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="49.6953125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.3359375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="14.6015625" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="10.0390625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="10.0390625" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="15.640625" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="10.609375" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="11.47265625" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" width="11.359375" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="18.34765625" customWidth="true" bestFit="true"/>
+    <col min="12" max="12" width="20.39453125" customWidth="true" bestFit="true"/>
+    <col min="13" max="13" width="7.30078125" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="36">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="36">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="35">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="35">
+        <v>156</v>
+      </c>
+      <c r="C3" t="s" s="35">
+        <v>157</v>
+      </c>
+      <c r="D3" t="s" s="35">
+        <v>207</v>
+      </c>
+      <c r="E3" t="s" s="35">
+        <v>208</v>
+      </c>
+      <c r="F3" t="s" s="35">
+        <v>209</v>
+      </c>
+      <c r="G3" t="s" s="35">
+        <v>162</v>
+      </c>
+      <c r="H3" t="s" s="35">
+        <v>210</v>
+      </c>
+      <c r="I3" t="s" s="35">
+        <v>164</v>
+      </c>
+      <c r="J3" t="s" s="35">
+        <v>166</v>
+      </c>
+      <c r="K3" t="s" s="35">
+        <v>167</v>
+      </c>
+      <c r="L3" t="s" s="35">
+        <v>168</v>
+      </c>
+      <c r="M3" t="s" s="35">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>211</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>212</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>213</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>214</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>184</v>
+      </c>
+      <c r="J4" t="s" s="0">
+        <v>179</v>
+      </c>
+      <c r="K4" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="L4" t="s" s="0">
+        <v>216</v>
+      </c>
+      <c r="M4" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="137.96875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="21.9609375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="6.4921875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="10.84375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="10.0390625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="10.0390625" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="23.41015625" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="16.90234375" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="18.60546875" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" width="8.1484375" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="7.90625" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="38">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="38">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="37">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="37">
+        <v>156</v>
+      </c>
+      <c r="C3" t="s" s="37">
+        <v>157</v>
+      </c>
+      <c r="D3" t="s" s="37">
+        <v>219</v>
+      </c>
+      <c r="E3" t="s" s="37">
+        <v>208</v>
+      </c>
+      <c r="F3" t="s" s="37">
+        <v>220</v>
+      </c>
+      <c r="G3" t="s" s="37">
+        <v>221</v>
+      </c>
+      <c r="H3" t="s" s="37">
+        <v>222</v>
+      </c>
+      <c r="I3" t="s" s="37">
+        <v>223</v>
+      </c>
+      <c r="J3" t="s" s="37">
+        <v>4</v>
+      </c>
+      <c r="K3" t="s" s="37">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>226</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>230</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="J4" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="K4" t="s" s="0">
+        <v>172</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:Q4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -1688,74 +2726,74 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="28">
+      <c r="A1" t="s" s="40">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="40">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="39">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="39">
+        <v>156</v>
+      </c>
+      <c r="C3" t="s" s="39">
+        <v>157</v>
+      </c>
+      <c r="D3" t="s" s="39">
+        <v>233</v>
+      </c>
+      <c r="E3" t="s" s="39">
+        <v>208</v>
+      </c>
+      <c r="F3" t="s" s="39">
+        <v>234</v>
+      </c>
+      <c r="G3" t="s" s="39">
+        <v>220</v>
+      </c>
+      <c r="H3" t="s" s="39">
+        <v>235</v>
+      </c>
+      <c r="I3" t="s" s="39">
+        <v>236</v>
+      </c>
+      <c r="J3" t="s" s="39">
+        <v>237</v>
+      </c>
+      <c r="K3" t="s" s="39">
+        <v>238</v>
+      </c>
+      <c r="L3" t="s" s="39">
+        <v>239</v>
+      </c>
+      <c r="M3" t="s" s="39">
+        <v>240</v>
+      </c>
+      <c r="N3" t="s" s="39">
+        <v>241</v>
+      </c>
+      <c r="O3" t="s" s="39">
+        <v>242</v>
+      </c>
+      <c r="P3" t="s" s="39">
+        <v>164</v>
+      </c>
+      <c r="Q3" t="s" s="39">
         <v>166</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="28">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="27">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s" s="27">
-        <v>117</v>
-      </c>
-      <c r="C3" t="s" s="27">
-        <v>118</v>
-      </c>
-      <c r="D3" t="s" s="27">
-        <v>168</v>
-      </c>
-      <c r="E3" t="s" s="27">
-        <v>169</v>
-      </c>
-      <c r="F3" t="s" s="27">
-        <v>170</v>
-      </c>
-      <c r="G3" t="s" s="27">
-        <v>171</v>
-      </c>
-      <c r="H3" t="s" s="27">
-        <v>172</v>
-      </c>
-      <c r="I3" t="s" s="27">
-        <v>173</v>
-      </c>
-      <c r="J3" t="s" s="27">
-        <v>174</v>
-      </c>
-      <c r="K3" t="s" s="27">
-        <v>175</v>
-      </c>
-      <c r="L3" t="s" s="27">
-        <v>176</v>
-      </c>
-      <c r="M3" t="s" s="27">
-        <v>177</v>
-      </c>
-      <c r="N3" t="s" s="27">
-        <v>178</v>
-      </c>
-      <c r="O3" t="s" s="27">
-        <v>179</v>
-      </c>
-      <c r="P3" t="s" s="27">
-        <v>125</v>
-      </c>
-      <c r="Q3" t="s" s="27">
-        <v>127</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>180</v>
+        <v>243</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>181</v>
+        <v>244</v>
       </c>
       <c r="C4" t="s" s="0">
         <v>6</v>
@@ -1764,377 +2802,43 @@
         <v>68</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>182</v>
+        <v>227</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>183</v>
+        <v>245</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>182</v>
+        <v>227</v>
       </c>
       <c r="H4" t="s" s="0">
-        <v>184</v>
+        <v>246</v>
       </c>
       <c r="I4" t="s" s="0">
-        <v>185</v>
+        <v>247</v>
       </c>
       <c r="J4" t="s" s="0">
-        <v>186</v>
+        <v>248</v>
       </c>
       <c r="K4" t="s" s="0">
         <v>26</v>
       </c>
       <c r="L4" t="s" s="0">
-        <v>187</v>
+        <v>249</v>
       </c>
       <c r="M4" t="s" s="0">
-        <v>140</v>
+        <v>179</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>140</v>
+        <v>179</v>
       </c>
       <c r="O4" t="s" s="0">
-        <v>137</v>
+        <v>176</v>
       </c>
       <c r="P4" t="s" s="0">
         <v>39</v>
       </c>
       <c r="Q4" t="s" s="0">
-        <v>140</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <cols>
-    <col min="1" max="1" width="99.8203125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="52.00390625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="10.3359375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="12.9296875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="14.02734375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="19.83984375" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="15.48046875" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="11.359375" customWidth="true" bestFit="true"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="30">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="30">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="29">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s" s="29">
-        <v>117</v>
-      </c>
-      <c r="C3" t="s" s="29">
-        <v>118</v>
-      </c>
-      <c r="D3" t="s" s="29">
-        <v>190</v>
-      </c>
-      <c r="E3" t="s" s="29">
-        <v>191</v>
-      </c>
-      <c r="F3" t="s" s="29">
-        <v>192</v>
-      </c>
-      <c r="G3" t="s" s="29">
-        <v>193</v>
-      </c>
-      <c r="H3" t="s" s="29">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>194</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>195</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>75</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>196</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>197</v>
-      </c>
-      <c r="G4" t="s" s="0">
-        <v>198</v>
-      </c>
-      <c r="H4" t="s" s="0">
-        <v>140</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <cols>
-    <col min="1" max="1" width="57.51171875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="22.40234375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="35.33984375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="7.07421875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="10.0390625" customWidth="true" bestFit="true"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="32">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="32">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="31">
-        <v>201</v>
-      </c>
-      <c r="B3" t="s" s="31">
-        <v>202</v>
-      </c>
-      <c r="C3" t="s" s="31">
-        <v>203</v>
-      </c>
-      <c r="D3" t="s" s="31">
-        <v>204</v>
-      </c>
-      <c r="E3" t="s" s="31">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>206</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>137</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>207</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>140</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>208</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>180</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>209</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>140</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>210</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>194</v>
-      </c>
-      <c r="C6" t="s" s="0">
-        <v>211</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>140</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <cols>
-    <col min="1" max="1" width="80.140625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="18.6953125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.296875" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="22.40234375" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="11.12890625" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="40.5625" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="12.12109375" customWidth="true" bestFit="true"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="34">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="34">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="33">
-        <v>214</v>
-      </c>
-      <c r="B3" t="s" s="33">
-        <v>215</v>
-      </c>
-      <c r="C3" t="s" s="33">
-        <v>216</v>
-      </c>
-      <c r="D3" t="s" s="33">
-        <v>217</v>
-      </c>
-      <c r="E3" t="s" s="33">
-        <v>218</v>
-      </c>
-      <c r="F3" t="s" s="33">
-        <v>117</v>
-      </c>
-      <c r="G3" t="s" s="33">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>210</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>194</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>206</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>137</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>220</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>221</v>
-      </c>
-      <c r="G4" t="s" s="0">
-        <v>13</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <cols>
-    <col min="1" max="1" width="51.7578125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="22.00390625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.42578125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="53.28125" customWidth="true" bestFit="true"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="36">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="36">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="35">
-        <v>201</v>
-      </c>
-      <c r="B3" t="s" s="35">
-        <v>202</v>
-      </c>
-      <c r="C3" t="s" s="35">
-        <v>224</v>
-      </c>
-      <c r="D3" t="s" s="35">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>206</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>131</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>226</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>208</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>180</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>226</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>210</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>194</v>
-      </c>
-      <c r="C6" t="s" s="0">
-        <v>226</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>227</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -2173,6 +2877,514 @@
     <row r="5">
       <c r="A5" t="s" s="0">
         <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="99.8203125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="52.00390625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.3359375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="12.9296875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="14.02734375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="19.83984375" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="15.48046875" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="11.359375" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="42">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="42">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="41">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="41">
+        <v>156</v>
+      </c>
+      <c r="C3" t="s" s="41">
+        <v>157</v>
+      </c>
+      <c r="D3" t="s" s="41">
+        <v>252</v>
+      </c>
+      <c r="E3" t="s" s="41">
+        <v>253</v>
+      </c>
+      <c r="F3" t="s" s="41">
+        <v>254</v>
+      </c>
+      <c r="G3" t="s" s="41">
+        <v>255</v>
+      </c>
+      <c r="H3" t="s" s="41">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>257</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>258</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>259</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>260</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>179</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="94.51953125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="41.515625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="6.4921875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="10.859375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="10.0390625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="7.5234375" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="11.359375" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="26.03515625" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="6.43359375" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="44">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="44">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="43">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="43">
+        <v>156</v>
+      </c>
+      <c r="C3" t="s" s="43">
+        <v>157</v>
+      </c>
+      <c r="D3" t="s" s="43">
+        <v>263</v>
+      </c>
+      <c r="E3" t="s" s="43">
+        <v>209</v>
+      </c>
+      <c r="F3" t="s" s="43">
+        <v>159</v>
+      </c>
+      <c r="G3" t="s" s="43">
+        <v>166</v>
+      </c>
+      <c r="H3" t="s" s="43">
+        <v>264</v>
+      </c>
+      <c r="I3" t="s" s="43">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>267</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>268</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>179</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>269</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="57.51171875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="53.28125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="45.37109375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="7.07421875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="10.0390625" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="46">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="46">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="45">
+        <v>272</v>
+      </c>
+      <c r="B3" t="s" s="45">
+        <v>273</v>
+      </c>
+      <c r="C3" t="s" s="45">
+        <v>274</v>
+      </c>
+      <c r="D3" t="s" s="45">
+        <v>275</v>
+      </c>
+      <c r="E3" t="s" s="45">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>176</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>179</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>243</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>179</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>281</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>179</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>211</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>179</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>285</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>286</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>179</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="80.140625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="32.15625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.296875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="53.28125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="11.12890625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="47.33203125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="12.12109375" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="48">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="48">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="47">
+        <v>289</v>
+      </c>
+      <c r="B3" t="s" s="47">
+        <v>290</v>
+      </c>
+      <c r="C3" t="s" s="47">
+        <v>291</v>
+      </c>
+      <c r="D3" t="s" s="47">
+        <v>292</v>
+      </c>
+      <c r="E3" t="s" s="47">
+        <v>293</v>
+      </c>
+      <c r="F3" t="s" s="47">
+        <v>156</v>
+      </c>
+      <c r="G3" t="s" s="47">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>281</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>176</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>295</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>296</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>285</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>211</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>297</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>298</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="51.7578125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="53.28125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.42578125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="53.28125" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="50">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="50">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="49">
+        <v>272</v>
+      </c>
+      <c r="B3" t="s" s="49">
+        <v>273</v>
+      </c>
+      <c r="C3" t="s" s="49">
+        <v>301</v>
+      </c>
+      <c r="D3" t="s" s="49">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>211</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>170</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>243</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>281</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>285</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>266</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -2949,14 +4161,16 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="92.55078125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="16.671875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="41.7109375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="20.73046875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="9.7734375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="77.05078125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="8.16015625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.109375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="5.51953125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="16.99609375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="13.42578125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="17.5703125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2966,7 +4180,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="18">
-        <v>80</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3">
@@ -2974,50 +4188,68 @@
         <v>2</v>
       </c>
       <c r="B3" t="s" s="17">
-        <v>81</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s" s="17">
-        <v>82</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s" s="17">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="E3" t="s" s="17">
-        <v>84</v>
+        <v>49</v>
+      </c>
+      <c r="F3" t="s" s="17">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s" s="17">
+        <v>21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>87</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>88</v>
+        <v>53</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>7</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>17</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>91</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>88</v>
+        <v>53</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>7</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>